<commit_message>
Update gold price tracking workbook
</commit_message>
<xml_diff>
--- a/gold_price_tracking.xlsx
+++ b/gold_price_tracking.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B109"/>
+  <dimension ref="A1:B110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.33203125" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -1477,6 +1477,16 @@
         <v>154908</v>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>152475</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>